<commit_message>
osworld: fix g9 replication bug, add closed-book/verify-replan harness, rerun affected sonnet5 tasks
Fixes a bug affecting g9 replication validity in osworld_eval.py and reruns
the subset of sonnet5 and verify-replan tasks affected by the fix and by
infra/rate-limit failures (113 of 303 task directories touched; legacy
pre-fix runs kept alongside for comparison). Adds the closed-book runner
and the codex_loop core module with tests, plus integration plans for the
longhorizon and verify-replan harnesses.
</commit_message>
<xml_diff>
--- a/benchmarks/osworld/results/agent_computer_sonnet5/51719eea-10bc-4246-a428-ac7c433dd4b3/run_1/BoomerangSales.xlsx
+++ b/benchmarks/osworld/results/agent_computer_sonnet5/51719eea-10bc-4246-a428-ac7c433dd4b3/run_1/BoomerangSales.xlsx
@@ -5,12 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Retail Price" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Retail Price" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <pivotCaches>
@@ -105,34 +105,34 @@
     <t xml:space="preserve">Sunset</t>
   </si>
   <si>
+    <t xml:space="preserve">Retail Price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alpine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carlota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Majestic Beaut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eagle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phoenix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Darnell Tri Fly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frido Fast Catch</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sum - Revenue</t>
   </si>
   <si>
     <t xml:space="preserve">Total Result</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retail Price</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alpine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carlota</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Majestic Beaut</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eagle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phoenix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Darnell Tri Fly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frido Fast Catch</t>
   </si>
 </sst>
 </file>
@@ -205,6 +205,13 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
       <left style="medium"/>
       <right style="thin"/>
       <top style="medium"/>
@@ -267,13 +274,6 @@
       <bottom style="medium"/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -327,48 +327,48 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="24" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="9" xfId="24" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="9" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1023,11 +1023,11 @@
         <v>0.165</v>
       </c>
       <c r="G2" s="0" t="n">
-        <f aca="false">VLOOKUP(C2,'Retail Price'!$A$2:$B$23,2,0)*E2*(1-F2)</f>
+        <f aca="false">VLOOKUP(C2,'Retail Price'!$A:$B,2,0)*E2*(1-F2)</f>
         <v>604.83225</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>42349.9764</v>
       </c>
@@ -1048,11 +1048,11 @@
         <v>0.15</v>
       </c>
       <c r="G3" s="0" t="n">
-        <f aca="false">VLOOKUP(C3,'Retail Price'!$A$2:$B$23,2,0)*E3*(1-F3)</f>
+        <f aca="false">VLOOKUP(C3,'Retail Price'!$A:$B,2,0)*E3*(1-F3)</f>
         <v>590.3675</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
         <v>42357.7576</v>
       </c>
@@ -1073,11 +1073,11 @@
         <v>0.019</v>
       </c>
       <c r="G4" s="0" t="n">
-        <f aca="false">VLOOKUP(C4,'Retail Price'!$A$2:$B$23,2,0)*E4*(1-F4)</f>
+        <f aca="false">VLOOKUP(C4,'Retail Price'!$A:$B,2,0)*E4*(1-F4)</f>
         <v>73.575</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
         <v>42239.5382</v>
       </c>
@@ -1098,11 +1098,11 @@
         <v>0.15</v>
       </c>
       <c r="G5" s="0" t="n">
-        <f aca="false">VLOOKUP(C5,'Retail Price'!$A$2:$B$23,2,0)*E5*(1-F5)</f>
+        <f aca="false">VLOOKUP(C5,'Retail Price'!$A:$B,2,0)*E5*(1-F5)</f>
         <v>1222.47</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
         <v>42194.2104</v>
       </c>
@@ -1123,11 +1123,11 @@
         <v>0.15</v>
       </c>
       <c r="G6" s="0" t="n">
-        <f aca="false">VLOOKUP(C6,'Retail Price'!$A$2:$B$23,2,0)*E6*(1-F6)</f>
+        <f aca="false">VLOOKUP(C6,'Retail Price'!$A:$B,2,0)*E6*(1-F6)</f>
         <v>579.785</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
         <v>42185.6951</v>
       </c>
@@ -1148,11 +1148,11 @@
         <v>0</v>
       </c>
       <c r="G7" s="0" t="n">
-        <f aca="false">VLOOKUP(C7,'Retail Price'!$A$2:$B$23,2,0)*E7*(1-F7)</f>
+        <f aca="false">VLOOKUP(C7,'Retail Price'!$A:$B,2,0)*E7*(1-F7)</f>
         <v>1000</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>42186.5528</v>
       </c>
@@ -1173,11 +1173,11 @@
         <v>0</v>
       </c>
       <c r="G8" s="0" t="n">
-        <f aca="false">VLOOKUP(C8,'Retail Price'!$A$2:$B$23,2,0)*E8*(1-F8)</f>
+        <f aca="false">VLOOKUP(C8,'Retail Price'!$A:$B,2,0)*E8*(1-F8)</f>
         <v>100</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
         <v>42218.1715</v>
       </c>
@@ -1198,11 +1198,11 @@
         <v>0.375</v>
       </c>
       <c r="G9" s="0" t="n">
-        <f aca="false">VLOOKUP(C9,'Retail Price'!$A$2:$B$23,2,0)*E9*(1-F9)</f>
+        <f aca="false">VLOOKUP(C9,'Retail Price'!$A:$B,2,0)*E9*(1-F9)</f>
         <v>1278.75</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
         <v>42324.5111</v>
       </c>
@@ -1223,11 +1223,11 @@
         <v>0.375</v>
       </c>
       <c r="G10" s="0" t="n">
-        <f aca="false">VLOOKUP(C10,'Retail Price'!$A$2:$B$23,2,0)*E10*(1-F10)</f>
+        <f aca="false">VLOOKUP(C10,'Retail Price'!$A:$B,2,0)*E10*(1-F10)</f>
         <v>560</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="n">
         <v>41982.825</v>
       </c>
@@ -1248,11 +1248,11 @@
         <v>0</v>
       </c>
       <c r="G11" s="0" t="n">
-        <f aca="false">VLOOKUP(C11,'Retail Price'!$A$2:$B$23,2,0)*E11*(1-F11)</f>
+        <f aca="false">VLOOKUP(C11,'Retail Price'!$A:$B,2,0)*E11*(1-F11)</f>
         <v>129</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
         <v>42346.3493</v>
       </c>
@@ -1273,11 +1273,11 @@
         <v>0.594</v>
       </c>
       <c r="G12" s="0" t="n">
-        <f aca="false">VLOOKUP(C12,'Retail Price'!$A$2:$B$23,2,0)*E12*(1-F12)</f>
+        <f aca="false">VLOOKUP(C12,'Retail Price'!$A:$B,2,0)*E12*(1-F12)</f>
         <v>2011.2428</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
         <v>41986.6875</v>
       </c>
@@ -1298,11 +1298,11 @@
         <v>0.15</v>
       </c>
       <c r="G13" s="0" t="n">
-        <f aca="false">VLOOKUP(C13,'Retail Price'!$A$2:$B$23,2,0)*E13*(1-F13)</f>
+        <f aca="false">VLOOKUP(C13,'Retail Price'!$A:$B,2,0)*E13*(1-F13)</f>
         <v>127.5</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="n">
         <v>42239.1299</v>
       </c>
@@ -1323,11 +1323,11 @@
         <v>0.072</v>
       </c>
       <c r="G14" s="0" t="n">
-        <f aca="false">VLOOKUP(C14,'Retail Price'!$A$2:$B$23,2,0)*E14*(1-F14)</f>
+        <f aca="false">VLOOKUP(C14,'Retail Price'!$A:$B,2,0)*E14*(1-F14)</f>
         <v>162.9568</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
         <v>42328.459</v>
       </c>
@@ -1348,11 +1348,11 @@
         <v>0.019</v>
       </c>
       <c r="G15" s="0" t="n">
-        <f aca="false">VLOOKUP(C15,'Retail Price'!$A$2:$B$23,2,0)*E15*(1-F15)</f>
+        <f aca="false">VLOOKUP(C15,'Retail Price'!$A:$B,2,0)*E15*(1-F15)</f>
         <v>294.3</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="n">
         <v>42242.4618</v>
       </c>
@@ -1373,11 +1373,11 @@
         <v>0.019</v>
       </c>
       <c r="G16" s="0" t="n">
-        <f aca="false">VLOOKUP(C16,'Retail Price'!$A$2:$B$23,2,0)*E16*(1-F16)</f>
+        <f aca="false">VLOOKUP(C16,'Retail Price'!$A:$B,2,0)*E16*(1-F16)</f>
         <v>64.59885</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="n">
         <v>42350.5986</v>
       </c>
@@ -1398,11 +1398,11 @@
         <v>0.356</v>
       </c>
       <c r="G17" s="0" t="n">
-        <f aca="false">VLOOKUP(C17,'Retail Price'!$A$2:$B$23,2,0)*E17*(1-F17)</f>
+        <f aca="false">VLOOKUP(C17,'Retail Price'!$A:$B,2,0)*E17*(1-F17)</f>
         <v>1286.3578</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="n">
         <v>41986.5278</v>
       </c>
@@ -1423,11 +1423,11 @@
         <v>0</v>
       </c>
       <c r="G18" s="0" t="n">
-        <f aca="false">VLOOKUP(C18,'Retail Price'!$A$2:$B$23,2,0)*E18*(1-F18)</f>
+        <f aca="false">VLOOKUP(C18,'Retail Price'!$A:$B,2,0)*E18*(1-F18)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
         <v>41985.691</v>
       </c>
@@ -1448,11 +1448,11 @@
         <v>0.159</v>
       </c>
       <c r="G19" s="0" t="n">
-        <f aca="false">VLOOKUP(C19,'Retail Price'!$A$2:$B$23,2,0)*E19*(1-F19)</f>
+        <f aca="false">VLOOKUP(C19,'Retail Price'!$A:$B,2,0)*E19*(1-F19)</f>
         <v>155.585</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
         <v>42213.6368</v>
       </c>
@@ -1473,11 +1473,11 @@
         <v>0</v>
       </c>
       <c r="G20" s="0" t="n">
-        <f aca="false">VLOOKUP(C20,'Retail Price'!$A$2:$B$23,2,0)*E20*(1-F20)</f>
+        <f aca="false">VLOOKUP(C20,'Retail Price'!$A:$B,2,0)*E20*(1-F20)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="n">
         <v>42241.6993</v>
       </c>
@@ -1498,11 +1498,11 @@
         <v>0.072</v>
       </c>
       <c r="G21" s="0" t="n">
-        <f aca="false">VLOOKUP(C21,'Retail Price'!$A$2:$B$23,2,0)*E21*(1-F21)</f>
+        <f aca="false">VLOOKUP(C21,'Retail Price'!$A:$B,2,0)*E21*(1-F21)</f>
         <v>122.2176</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="n">
         <v>42358.5243</v>
       </c>
@@ -1523,11 +1523,11 @@
         <v>0.16</v>
       </c>
       <c r="G22" s="0" t="n">
-        <f aca="false">VLOOKUP(C22,'Retail Price'!$A$2:$B$23,2,0)*E22*(1-F22)</f>
+        <f aca="false">VLOOKUP(C22,'Retail Price'!$A:$B,2,0)*E22*(1-F22)</f>
         <v>147</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="n">
         <v>42245.5875</v>
       </c>
@@ -1548,11 +1548,11 @@
         <v>0.019</v>
       </c>
       <c r="G23" s="0" t="n">
-        <f aca="false">VLOOKUP(C23,'Retail Price'!$A$2:$B$23,2,0)*E23*(1-F23)</f>
+        <f aca="false">VLOOKUP(C23,'Retail Price'!$A:$B,2,0)*E23*(1-F23)</f>
         <v>117.72</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="n">
         <v>42063.4896</v>
       </c>
@@ -1573,11 +1573,11 @@
         <v>0</v>
       </c>
       <c r="G24" s="0" t="n">
-        <f aca="false">VLOOKUP(C24,'Retail Price'!$A$2:$B$23,2,0)*E24*(1-F24)</f>
+        <f aca="false">VLOOKUP(C24,'Retail Price'!$A:$B,2,0)*E24*(1-F24)</f>
         <v>129</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="n">
         <v>42198.2292</v>
       </c>
@@ -1598,11 +1598,11 @@
         <v>0.169</v>
       </c>
       <c r="G25" s="0" t="n">
-        <f aca="false">VLOOKUP(C25,'Retail Price'!$A$2:$B$23,2,0)*E25*(1-F25)</f>
+        <f aca="false">VLOOKUP(C25,'Retail Price'!$A:$B,2,0)*E25*(1-F25)</f>
         <v>565.08</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="n">
         <v>42230.4097</v>
       </c>
@@ -1623,11 +1623,11 @@
         <v>0</v>
       </c>
       <c r="G26" s="0" t="n">
-        <f aca="false">VLOOKUP(C26,'Retail Price'!$A$2:$B$23,2,0)*E26*(1-F26)</f>
+        <f aca="false">VLOOKUP(C26,'Retail Price'!$A:$B,2,0)*E26*(1-F26)</f>
         <v>66</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="n">
         <v>42335.4819</v>
       </c>
@@ -1648,11 +1648,11 @@
         <v>0</v>
       </c>
       <c r="G27" s="0" t="n">
-        <f aca="false">VLOOKUP(C27,'Retail Price'!$A$2:$B$23,2,0)*E27*(1-F27)</f>
+        <f aca="false">VLOOKUP(C27,'Retail Price'!$A:$B,2,0)*E27*(1-F27)</f>
         <v>24</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="n">
         <v>42311.5215</v>
       </c>
@@ -1673,11 +1673,11 @@
         <v>0.071</v>
       </c>
       <c r="G28" s="0" t="n">
-        <f aca="false">VLOOKUP(C28,'Retail Price'!$A$2:$B$23,2,0)*E28*(1-F28)</f>
+        <f aca="false">VLOOKUP(C28,'Retail Price'!$A:$B,2,0)*E28*(1-F28)</f>
         <v>23.225</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="n">
         <v>42103.5299</v>
       </c>
@@ -1698,11 +1698,11 @@
         <v>0.375</v>
       </c>
       <c r="G29" s="0" t="n">
-        <f aca="false">VLOOKUP(C29,'Retail Price'!$A$2:$B$23,2,0)*E29*(1-F29)</f>
+        <f aca="false">VLOOKUP(C29,'Retail Price'!$A:$B,2,0)*E29*(1-F29)</f>
         <v>1105</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="n">
         <v>42346.7611</v>
       </c>
@@ -1723,11 +1723,11 @@
         <v>0</v>
       </c>
       <c r="G30" s="0" t="n">
-        <f aca="false">VLOOKUP(C30,'Retail Price'!$A$2:$B$23,2,0)*E30*(1-F30)</f>
+        <f aca="false">VLOOKUP(C30,'Retail Price'!$A:$B,2,0)*E30*(1-F30)</f>
         <v>20</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="n">
         <v>42054.9257</v>
       </c>
@@ -1748,11 +1748,11 @@
         <v>0</v>
       </c>
       <c r="G31" s="0" t="n">
-        <f aca="false">VLOOKUP(C31,'Retail Price'!$A$2:$B$23,2,0)*E31*(1-F31)</f>
+        <f aca="false">VLOOKUP(C31,'Retail Price'!$A:$B,2,0)*E31*(1-F31)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="n">
         <v>42350.3646</v>
       </c>
@@ -1773,11 +1773,11 @@
         <v>0</v>
       </c>
       <c r="G32" s="0" t="n">
-        <f aca="false">VLOOKUP(C32,'Retail Price'!$A$2:$B$23,2,0)*E32*(1-F32)</f>
+        <f aca="false">VLOOKUP(C32,'Retail Price'!$A:$B,2,0)*E32*(1-F32)</f>
         <v>75</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="n">
         <v>41982.5083</v>
       </c>
@@ -1798,11 +1798,11 @@
         <v>0</v>
       </c>
       <c r="G33" s="0" t="n">
-        <f aca="false">VLOOKUP(C33,'Retail Price'!$A$2:$B$23,2,0)*E33*(1-F33)</f>
+        <f aca="false">VLOOKUP(C33,'Retail Price'!$A:$B,2,0)*E33*(1-F33)</f>
         <v>21.95</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="n">
         <v>41980.8229</v>
       </c>
@@ -1823,11 +1823,11 @@
         <v>0.018</v>
       </c>
       <c r="G34" s="0" t="n">
-        <f aca="false">VLOOKUP(C34,'Retail Price'!$A$2:$B$23,2,0)*E34*(1-F34)</f>
+        <f aca="false">VLOOKUP(C34,'Retail Price'!$A:$B,2,0)*E34*(1-F34)</f>
         <v>220.95</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="n">
         <v>41979.7403</v>
       </c>
@@ -1848,11 +1848,11 @@
         <v>0.019</v>
       </c>
       <c r="G35" s="0" t="n">
-        <f aca="false">VLOOKUP(C35,'Retail Price'!$A$2:$B$23,2,0)*E35*(1-F35)</f>
+        <f aca="false">VLOOKUP(C35,'Retail Price'!$A:$B,2,0)*E35*(1-F35)</f>
         <v>4.905</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="n">
         <v>42158.1625</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>0</v>
       </c>
       <c r="G36" s="0" t="n">
-        <f aca="false">VLOOKUP(C36,'Retail Price'!$A$2:$B$23,2,0)*E36*(1-F36)</f>
+        <f aca="false">VLOOKUP(C36,'Retail Price'!$A:$B,2,0)*E36*(1-F36)</f>
         <v>71.8</v>
       </c>
     </row>
@@ -1893,142 +1893,349 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr defaultColWidth="8.515625" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.89"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>21.95</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>21.95</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>19.95</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>17.95</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>26.95</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>21.95</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>23.95</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>23.95</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>9.95</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>39.95</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B17"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>26</v>
+      <c r="B1" s="5" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="5" t="n">
+      <c r="B2" s="7" t="n">
         <v>2262.9133</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="7" t="n">
+      <c r="B3" s="9" t="n">
         <v>173.575</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="7" t="n">
+      <c r="B4" s="9" t="n">
         <v>258</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="9" t="n">
         <v>590.25</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="9" t="n">
         <v>651.585</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="9" t="n">
         <v>1344.75</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="9" t="n">
         <v>508.215</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="9" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="9" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="9" t="n">
         <v>117.72</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="9" t="n">
         <v>3233.7128</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="9" t="n">
         <v>1105</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="9" t="n">
         <v>565.08</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
         <v>560</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="10" t="n">
         <v>590.3675</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="10" t="n">
+      <c r="A17" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="12" t="n">
         <v>12985.1686</v>
       </c>
     </row>
@@ -2041,211 +2248,4 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:B23"/>
-  <sheetFormatPr defaultColWidth="8.515625" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.89"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B2" s="12" t="n">
-        <v>21.95</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="12" t="n">
-        <v>21.95</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="12" t="n">
-        <v>19.95</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="12" t="n">
-        <v>17.95</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="12" t="n">
-        <v>26.95</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="12" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="12" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="12" t="n">
-        <v>21.95</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="12" t="n">
-        <v>23.95</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="12" t="n">
-        <v>23.95</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="12" t="n">
-        <v>9.95</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="12" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" s="12" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" s="12" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="12" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="12" t="n">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="12" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="B19" s="12" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20" s="12" t="n">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B21" s="12" t="n">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="B22" s="12" t="n">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B23" s="12" t="n">
-        <v>39.95</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>